<commit_message>
Regenerate structural metrics and publication figures with sigma0-fixed CMA-ES results
All 120 CMA-ES cases (6 scenarios x 20 test cases) were rerun with the
sigma0 normalization fix (previous commit). This regenerates the
downstream structural evaluation and publication outputs from those
results:

- calibration/comparison_structure_metrics_v2_*.csv (all 6 modes,
  via evaluate_ml_structure_unified.jl)
- Table 1 (now N=20 for S1 instead of N=18 — A_497 and C_100 are no
  longer excluded, since both now have completed CMA-ES-S1MS fits)
- Figures 3, 4, 5, S2, S3

Notably, Figure 5 no longer shows CMA-ES-S1 accuracy decreasing with
observation seed count k — SS_rld and SS_angle now both increase
monotonically with k, consistent with every other series in the plot.
This confirms the sigma0 scaling bug was the cause of that anomaly.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/publication/figures/table1_structural.xlsx
+++ b/publication/figures/table1_structural.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Table1_v2" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Table1_v2" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -536,16 +536,16 @@
         </is>
       </c>
       <c r="C2" s="3" t="n">
-        <v>-0.024</v>
+        <v>0.089</v>
       </c>
       <c r="D2" s="3" t="n">
-        <v>0.6840000000000001</v>
+        <v>0.485</v>
       </c>
       <c r="E2" s="3" t="n">
-        <v>0.101</v>
+        <v>0.065</v>
       </c>
       <c r="F2" s="3" t="n">
-        <v>0.453</v>
+        <v>0.508</v>
       </c>
       <c r="G2" s="3" t="n">
         <v>20</v>
@@ -565,16 +565,16 @@
         </is>
       </c>
       <c r="C3" s="4" t="n">
-        <v>0.128</v>
+        <v>0.134</v>
       </c>
       <c r="D3" s="3" t="n">
-        <v>0.91</v>
+        <v>0.905</v>
       </c>
       <c r="E3" s="4" t="n">
-        <v>0.393</v>
+        <v>0.417</v>
       </c>
       <c r="F3" s="3" t="n">
-        <v>0.375</v>
+        <v>0.359</v>
       </c>
       <c r="G3" s="3" t="n">
         <v>20</v>
@@ -598,19 +598,19 @@
         </is>
       </c>
       <c r="C4" s="4" t="n">
-        <v>-0.068</v>
+        <v>0.27</v>
       </c>
       <c r="D4" s="3" t="n">
-        <v>0.614</v>
+        <v>0.367</v>
       </c>
       <c r="E4" s="3" t="n">
-        <v>-0.139</v>
+        <v>-0.04</v>
       </c>
       <c r="F4" s="3" t="n">
-        <v>0.707</v>
+        <v>0.74</v>
       </c>
       <c r="G4" s="3" t="n">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="H4" s="3" t="b">
         <v>1</v>
@@ -627,19 +627,19 @@
         </is>
       </c>
       <c r="C5" s="3" t="n">
-        <v>-0.101</v>
+        <v>-0.018</v>
       </c>
       <c r="D5" s="3" t="n">
-        <v>1.195</v>
+        <v>1.15</v>
       </c>
       <c r="E5" s="4" t="n">
-        <v>0.26</v>
+        <v>0.298</v>
       </c>
       <c r="F5" s="3" t="n">
-        <v>0.445</v>
+        <v>0.413</v>
       </c>
       <c r="G5" s="3" t="n">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="H5" s="3" t="b">
         <v>0</v>
@@ -651,7 +651,7 @@
     <row r="7">
       <c r="A7" s="6" t="inlineStr">
         <is>
-          <t>Notes: skin_depth = 0.2 cm (2 mm), k = 7 seeds. SS &gt; 0 = better than null predictor. Bold = best per scenario. S2: elongation known, 4 arch params. S1: all 8 params unknown. S1 N=18 (A_497 and C_100 excluded from S1 calibration).</t>
+          <t>Notes: skin_depth = 0.2 cm (2 mm), k = 7 seeds. SS &gt; 0 = better than null predictor. Bold = best per scenario. S2: elongation known, 4 arch params. S1: all 8 params unknown.</t>
         </is>
       </c>
     </row>

</xml_diff>